<commit_message>
Ship compliance workflows and demo seed
</commit_message>
<xml_diff>
--- a/market-research/Leasium_Market_Sizing.xlsx
+++ b/market-research/Leasium_Market_Sizing.xlsx
@@ -93,7 +93,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="295">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="299">
   <si>
     <t xml:space="preserve">Leasium — SMB Property Manager Market Sizing</t>
   </si>
@@ -167,7 +167,7 @@
     <t xml:space="preserve">• See the per-country tabs for the build-up and the 'Sources &amp; Notes' tab for citations, confidence and caveats.</t>
   </si>
   <si>
-    <t xml:space="preserve">Leasium — Scaled Targets, Revenue &amp; Pricing</t>
+    <t xml:space="preserve">Leasium — Phased Targets, Revenue &amp; Pricing</t>
   </si>
   <si>
     <t xml:space="preserve">1. Pricing (per tenant / month)</t>
@@ -176,229 +176,241 @@
     <t xml:space="preserve">Private PM — self-managing landlords</t>
   </si>
   <si>
-    <t xml:space="preserve">Higher volume / lower touch → lower price</t>
-  </si>
-  <si>
     <t xml:space="preserve">SMB property managers — smaller</t>
   </si>
   <si>
     <t xml:space="preserve">SMB property managers — larger</t>
   </si>
   <si>
-    <t xml:space="preserve">Blended ARPU (base case)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Editable — mix of private vs agency tenants</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. Scaled targets (tenants on platform)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brisbane</t>
+    <t xml:space="preserve">Blended ARPU — landing phases (1-3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blended ARPU — PM expansion (Phase 4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agency pricing — Phase 4 is property managers ($3-4).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Phased targets &amp; revenue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phase</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tenants</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARPU/mo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MRR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% of market</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phase 1 — Brisbane</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phase 2 — SE Queensland</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phase 3 — National (AU)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phase 4 — PM-business expansion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% of market: phases 1-3 = share of total rentals in that geography; Phase 4 = share of the national agent-managed (agency) market (~2.0M doors).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Phase 4 expansion — ARR sensitivity (500,000 tenancies)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agency ARPU / month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$3.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$3.50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$4.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Annual recurring revenue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Competitor cost reference (effective $/unit/month, small portfolio)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Product</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$/unit/mo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Segment / note</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leasium — private landlords</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Self-managing landlords</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leasium — SMB agency (small)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Small agencies</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leasium — SMB agency (large)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Larger agencies</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RentBetter (AU)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Self-managing landlord app — $29-36/property</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RentingSmart (AU)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Self-managing landlord app — $15-25/property</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PropertyMe (AU)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agency PM; from $1.76/prop at 100 (~$8.80 at 20, $176 floor)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DoorLoop (US)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Per-unit w/ plan floor: Starter $69/mo (&lt;=10 units) = $6.90/unit; ~$3/unit at volume</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hemlane (US)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$36.50 base + $2.50/unit (at 20 units)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buildium (US)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">From $58/mo; scales ~$2-3/unit at volume</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TenantCloud (US)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">From $17/mo; free tier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Re-Leased (commercial)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quote-based; ~$18-72/unit at 5-20 units incl. floor+setup</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Effective $/unit at a small portfolio. AU tools priced per property; US tools scale (plan floor small -&gt; ~$2-3/unit at volume). Re-Leased quote-based (estimated). Sources: vendor sites + Capterra/GetApp.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SE Queensland — Brisbane launch → SEQ rollout</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anchored on the RTA's hard bond count (631,805 QLD tenancies, Jun 2025). Brisbane = beachhead; SEQ = the rollout. Segment ratios reuse the Australia tab; maintenance layer added for partner-building.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assumptions (edit blue cells; green cells link to the Australia tab)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QLD active rental bonds (RTA, 30 Jun 2025)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source: RTA Annual Report 2024-25 (~$1.3B held).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Greater Brisbane share of QLD bonds</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apportionment, anchored to ~48% pop / ~50% rental share. Refine w/ RTA LGA data.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SE Queensland share of QLD bonds</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apportionment, anchored to ~71% pop / higher urban rental share.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Self-management rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Linked from Australia tab (30%). QLD may run higher.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Multi-property share of rental dwellings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">From ATO: multi-property investors hold ~51% of dwellings.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avg dwellings per multi-property landlord</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Linked from Australia tab (~2.3).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agent-managed rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equals 1 minus the self-management rate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Median weekly rent (SEQ, RTA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RTA Q2-2025: Brisbane combined ~$625-700/wk; SEQ blend conservative.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maintenance as % of annual rent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Industry rule of thumb 5-10% of gross rent.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maintenance jobs per tenancy / year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Planning estimate: reactive + periodic jobs per rental/yr.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QLD construction businesses (ABS)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ABS Counts of Australian Businesses; QLD construction ~17% of 511,835.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maintenance-relevant trades share</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Est. share of construction firms doing rental maintenance trades.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Greater Brisbane</t>
   </si>
   <si>
     <t xml:space="preserve">SE Queensland</t>
-  </si>
-  <si>
-    <t xml:space="preserve">National (AU)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Phase</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Target tenants</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 → 2 → 3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MRR @ blended ($)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARR @ blended ($)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARR @ $5 (all private)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARR @ $4 (blended)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARR @ $3 (all large agency)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Target as % of TOTAL rental market</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Target as % of self-managing 2-20 segment</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US = Phase 4 (separate model)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. Competitor cost reference (effective $/unit/month, small portfolio)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Product</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$/unit/mo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Segment / note</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Leasium — private landlords</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Self-managing landlords</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Leasium — SMB agency (small)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Small agencies</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Leasium — SMB agency (large)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Larger agencies</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RentBetter (AU)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Self-managing landlord app — $29-36/property</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RentingSmart (AU)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Self-managing landlord app — $15-25/property</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PropertyMe (AU)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Agency PM; from $1.76/prop at 100 (≈$8.80 at 20, $176 floor)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DoorLoop (US)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Per-unit w/ plan floor: Starter $69/mo (&lt;=10 units) = $6.90/unit; scales toward ~$3/unit at volume</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Buildium (US)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">From $58/mo; ~$2.40/unit at 100</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hemlane (US)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$36.50 base + $2.50/unit (at 20 units)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TenantCloud (US)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">From $17/mo; free tier</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Re-Leased (commercial)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quote-based; ~$18-72/unit at 5-20 units incl. floor+setup</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Competitor prices are published list/entry pricing converted to an effective per-unit rate at a small portfolio; AU tools priced per property, US per unit. Re-Leased is quote-based (estimated). Sources on respective sites + Capterra/GetApp.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SE Queensland — Brisbane launch → SEQ rollout</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Anchored on the RTA's hard bond count (631,805 QLD tenancies, Jun 2025). Brisbane = beachhead; SEQ = the rollout. Segment ratios reuse the Australia tab; maintenance layer added for partner-building.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Assumptions (edit blue cells; green cells link to the Australia tab)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">QLD active rental bonds (RTA, 30 Jun 2025)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Source: RTA Annual Report 2024-25 (~$1.3B held).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Greater Brisbane share of QLD bonds</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Apportionment, anchored to ~48% pop / ~50% rental share. Refine w/ RTA LGA data.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SE Queensland share of QLD bonds</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Apportionment, anchored to ~71% pop / higher urban rental share.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Self-management rate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Linked from Australia tab (30%). QLD may run higher.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Multi-property share of rental dwellings</t>
-  </si>
-  <si>
-    <t xml:space="preserve">From ATO: multi-property investors hold ~51% of dwellings.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Avg dwellings per multi-property landlord</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Linked from Australia tab (~2.3).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Agent-managed rate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Equals 1 minus the self-management rate.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Median weekly rent (SEQ, RTA)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RTA Q2-2025: Brisbane combined ~$625-700/wk; SEQ blend conservative.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Maintenance as % of annual rent</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Industry rule of thumb 5-10% of gross rent.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Maintenance jobs per tenancy / year</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Planning estimate: reactive + periodic jobs per rental/yr.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">QLD construction businesses (ABS)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ABS Counts of Australian Businesses; QLD construction ~17% of 511,835.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Maintenance-relevant trades share</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Est. share of construction firms doing rental maintenance trades.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Greater Brisbane</t>
   </si>
   <si>
     <t xml:space="preserve">Queensland</t>
@@ -995,7 +1007,7 @@
     <numFmt numFmtId="171" formatCode="\$#,##0;&quot;($&quot;#,##0\);\-"/>
     <numFmt numFmtId="172" formatCode="0.00"/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="25">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1103,9 +1115,9 @@
       <charset val="1"/>
     </font>
     <font>
-      <i val="true"/>
+      <b val="true"/>
       <sz val="9"/>
-      <color rgb="FF000000"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -1136,14 +1148,6 @@
     <font>
       <sz val="9"/>
       <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="9"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -1277,7 +1281,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="76">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1346,91 +1350,111 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="17" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="171" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="171" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="17" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="172" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="20" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1470,7 +1494,7 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1478,7 +1502,7 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1522,7 +1546,7 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="24" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="23" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1546,11 +1570,11 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="24" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="23" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1558,7 +1582,7 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2130,11 +2154,15 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2145,6 +2173,7 @@
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
@@ -2154,6 +2183,7 @@
       <c r="C3" s="14"/>
       <c r="D3" s="14"/>
       <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
@@ -2162,15 +2192,10 @@
       <c r="B4" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="C4" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B5" s="15" t="n">
         <v>4</v>
@@ -2178,7 +2203,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B6" s="15" t="n">
         <v>3</v>
@@ -2186,55 +2211,53 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B7" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="C7" s="16" t="s">
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" s="15" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="C8" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="D7" s="16"/>
-      <c r="E7" s="16"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="14" t="s">
+      <c r="D8" s="16"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="16"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="B9" s="14"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="17"/>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="14"/>
+      <c r="C10" s="14"/>
+      <c r="D10" s="14"/>
+      <c r="E10" s="14"/>
+      <c r="F10" s="14"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="C10" s="18" t="s">
+      <c r="B11" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="D10" s="18" t="s">
+      <c r="C11" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="E10" s="18" t="s">
+      <c r="D11" s="17" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="19" t="s">
+      <c r="E11" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="B11" s="20" t="n">
-        <v>5000</v>
-      </c>
-      <c r="C11" s="20" t="n">
-        <v>10000</v>
-      </c>
-      <c r="D11" s="20" t="n">
-        <v>100000</v>
-      </c>
-      <c r="E11" s="21" t="s">
+      <c r="F11" s="17" t="s">
         <v>38</v>
       </c>
     </row>
@@ -2242,329 +2265,362 @@
       <c r="A12" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="B12" s="22" t="n">
-        <f aca="false">B11*$B$7</f>
+      <c r="B12" s="18" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C12" s="19" t="n">
+        <f aca="false">$B$7</f>
+        <v>4</v>
+      </c>
+      <c r="D12" s="20" t="n">
+        <f aca="false">B12*C12</f>
         <v>20000</v>
       </c>
-      <c r="C12" s="22" t="n">
-        <f aca="false">C11*$B$7</f>
+      <c r="E12" s="21" t="n">
+        <f aca="false">D12*12</f>
+        <v>240000</v>
+      </c>
+      <c r="F12" s="22" t="n">
+        <f aca="false">B12/'SE Queensland'!B20</f>
+        <v>0.0158276683470375</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B13" s="18" t="n">
+        <v>10000</v>
+      </c>
+      <c r="C13" s="19" t="n">
+        <f aca="false">$B$7</f>
+        <v>4</v>
+      </c>
+      <c r="D13" s="20" t="n">
+        <f aca="false">B13*C13</f>
         <v>40000</v>
       </c>
-      <c r="D12" s="22" t="n">
-        <f aca="false">D11*$B$7</f>
-        <v>400000</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="19" t="s">
-        <v>40</v>
-      </c>
-      <c r="B13" s="23" t="n">
-        <f aca="false">B11*$B$7*12</f>
-        <v>240000</v>
-      </c>
-      <c r="C13" s="23" t="n">
-        <f aca="false">C11*$B$7*12</f>
+      <c r="E13" s="21" t="n">
+        <f aca="false">D13*12</f>
         <v>480000</v>
       </c>
-      <c r="D13" s="23" t="n">
-        <f aca="false">D11*$B$7*12</f>
-        <v>4800000</v>
+      <c r="F13" s="22" t="n">
+        <f aca="false">B13/'SE Queensland'!C20</f>
+        <v>0.0216817374616951</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B14" s="22" t="n">
-        <f aca="false">B11*$B$4*12</f>
-        <v>300000</v>
-      </c>
-      <c r="C14" s="22" t="n">
-        <f aca="false">C11*$B$4*12</f>
-        <v>600000</v>
-      </c>
-      <c r="D14" s="22" t="n">
-        <f aca="false">D11*$B$4*12</f>
-        <v>6000000</v>
+      <c r="B14" s="18" t="n">
+        <v>100000</v>
+      </c>
+      <c r="C14" s="19" t="n">
+        <f aca="false">$B$7</f>
+        <v>4</v>
+      </c>
+      <c r="D14" s="20" t="n">
+        <f aca="false">B14*C14</f>
+        <v>400000</v>
+      </c>
+      <c r="E14" s="21" t="n">
+        <f aca="false">D14*12</f>
+        <v>4800000</v>
+      </c>
+      <c r="F14" s="22" t="n">
+        <f aca="false">B14/Australia!B17</f>
+        <v>0.0344827586206897</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="s">
+      <c r="A15" s="23" t="s">
         <v>42</v>
       </c>
-      <c r="B15" s="22" t="n">
-        <f aca="false">B11*$B$5*12</f>
-        <v>240000</v>
-      </c>
-      <c r="C15" s="22" t="n">
-        <f aca="false">C11*$B$5*12</f>
-        <v>480000</v>
-      </c>
-      <c r="D15" s="22" t="n">
-        <f aca="false">D11*$B$5*12</f>
-        <v>4800000</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5" t="s">
+      <c r="B15" s="18" t="n">
+        <v>500000</v>
+      </c>
+      <c r="C15" s="19" t="n">
+        <f aca="false">$B$8</f>
+        <v>3.5</v>
+      </c>
+      <c r="D15" s="20" t="n">
+        <f aca="false">B15*C15</f>
+        <v>1750000</v>
+      </c>
+      <c r="E15" s="24" t="n">
+        <f aca="false">D15*12</f>
+        <v>21000000</v>
+      </c>
+      <c r="F15" s="22" t="n">
+        <f aca="false">B15/Australia!B34</f>
+        <v>0.246305418719212</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="25" t="s">
         <v>43</v>
       </c>
-      <c r="B16" s="22" t="n">
-        <f aca="false">B11*$B$6*12</f>
-        <v>180000</v>
-      </c>
-      <c r="C16" s="22" t="n">
-        <f aca="false">C11*$B$6*12</f>
-        <v>360000</v>
-      </c>
-      <c r="D16" s="22" t="n">
-        <f aca="false">D11*$B$6*12</f>
-        <v>3600000</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5" t="s">
+      <c r="B16" s="25"/>
+      <c r="C16" s="25"/>
+      <c r="D16" s="25"/>
+      <c r="E16" s="25"/>
+      <c r="F16" s="25"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="B17" s="24" t="n">
-        <f aca="false">B11/'SE Queensland'!B20</f>
-        <v>0.0158276683470375</v>
-      </c>
-      <c r="C17" s="24" t="n">
-        <f aca="false">C11/'SE Queensland'!C20</f>
-        <v>0.0216817374616951</v>
-      </c>
-      <c r="D17" s="24" t="n">
-        <f aca="false">D11/Australia!B17</f>
-        <v>0.0344827586206897</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5" t="s">
+      <c r="B18" s="14"/>
+      <c r="C18" s="14"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="14"/>
+      <c r="F18" s="14"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="23" t="s">
         <v>45</v>
       </c>
-      <c r="B18" s="24" t="n">
-        <f aca="false">B11/'SE Queensland'!B25</f>
-        <v>0.103448812725735</v>
-      </c>
-      <c r="C18" s="24" t="n">
-        <f aca="false">C11/'SE Queensland'!C25</f>
-        <v>0.141710702364021</v>
-      </c>
-      <c r="D18" s="24" t="n">
-        <f aca="false">D11/Australia!B28</f>
-        <v>0.223993882422439</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="16" t="s">
+      <c r="B19" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="B19" s="16"/>
-      <c r="C19" s="16"/>
-      <c r="D19" s="16"/>
-      <c r="E19" s="16"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="14" t="s">
+      <c r="C19" s="26" t="s">
         <v>47</v>
       </c>
-      <c r="B21" s="14"/>
-      <c r="C21" s="14"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="14"/>
+      <c r="D19" s="26" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="B20" s="27" t="n">
+        <f aca="false">500000*3*12</f>
+        <v>18000000</v>
+      </c>
+      <c r="C20" s="28" t="n">
+        <f aca="false">500000*3.5*12</f>
+        <v>21000000</v>
+      </c>
+      <c r="D20" s="27" t="n">
+        <f aca="false">500000*4*12</f>
+        <v>24000000</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="25" t="s">
-        <v>48</v>
-      </c>
-      <c r="B22" s="18" t="s">
-        <v>49</v>
-      </c>
-      <c r="C22" s="25" t="s">
+      <c r="A22" s="14" t="s">
         <v>50</v>
       </c>
-      <c r="D22" s="25"/>
-      <c r="E22" s="25"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="26" t="s">
+      <c r="B22" s="14"/>
+      <c r="C22" s="14"/>
+      <c r="D22" s="14"/>
+      <c r="E22" s="14"/>
+      <c r="F22" s="14"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="29" t="s">
         <v>51</v>
       </c>
-      <c r="B23" s="27" t="n">
+      <c r="B23" s="30" t="s">
+        <v>52</v>
+      </c>
+      <c r="C23" s="29" t="s">
+        <v>53</v>
+      </c>
+      <c r="D23" s="29"/>
+      <c r="E23" s="29"/>
+      <c r="F23" s="29"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="31" t="s">
+        <v>54</v>
+      </c>
+      <c r="B24" s="32" t="n">
         <f aca="false">B4</f>
         <v>5</v>
       </c>
-      <c r="C23" s="28" t="s">
-        <v>52</v>
-      </c>
-      <c r="D23" s="28"/>
-      <c r="E23" s="28"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="26" t="s">
-        <v>53</v>
-      </c>
-      <c r="B24" s="27" t="n">
+      <c r="C24" s="33" t="s">
+        <v>55</v>
+      </c>
+      <c r="D24" s="33"/>
+      <c r="E24" s="33"/>
+      <c r="F24" s="33"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="31" t="s">
+        <v>56</v>
+      </c>
+      <c r="B25" s="32" t="n">
         <f aca="false">B5</f>
         <v>4</v>
       </c>
-      <c r="C24" s="28" t="s">
-        <v>54</v>
-      </c>
-      <c r="D24" s="28"/>
-      <c r="E24" s="28"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="26" t="s">
-        <v>55</v>
-      </c>
-      <c r="B25" s="27" t="n">
+      <c r="C25" s="33" t="s">
+        <v>57</v>
+      </c>
+      <c r="D25" s="33"/>
+      <c r="E25" s="33"/>
+      <c r="F25" s="33"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="31" t="s">
+        <v>58</v>
+      </c>
+      <c r="B26" s="32" t="n">
         <f aca="false">B6</f>
         <v>3</v>
       </c>
-      <c r="C25" s="28" t="s">
-        <v>56</v>
-      </c>
-      <c r="D25" s="28"/>
-      <c r="E25" s="28"/>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="29" t="s">
-        <v>57</v>
-      </c>
-      <c r="B26" s="30" t="n">
+      <c r="C26" s="33" t="s">
+        <v>59</v>
+      </c>
+      <c r="D26" s="33"/>
+      <c r="E26" s="33"/>
+      <c r="F26" s="33"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="34" t="s">
+        <v>60</v>
+      </c>
+      <c r="B27" s="35" t="n">
         <v>32</v>
       </c>
-      <c r="C26" s="28" t="s">
-        <v>58</v>
-      </c>
-      <c r="D26" s="28"/>
-      <c r="E26" s="28"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="29" t="s">
-        <v>59</v>
-      </c>
-      <c r="B27" s="30" t="n">
+      <c r="C27" s="33" t="s">
+        <v>61</v>
+      </c>
+      <c r="D27" s="33"/>
+      <c r="E27" s="33"/>
+      <c r="F27" s="33"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="34" t="s">
+        <v>62</v>
+      </c>
+      <c r="B28" s="35" t="n">
         <v>20</v>
       </c>
-      <c r="C27" s="28" t="s">
-        <v>60</v>
-      </c>
-      <c r="D27" s="28"/>
-      <c r="E27" s="28"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="29" t="s">
-        <v>61</v>
-      </c>
-      <c r="B28" s="30" t="n">
+      <c r="C28" s="33" t="s">
+        <v>63</v>
+      </c>
+      <c r="D28" s="33"/>
+      <c r="E28" s="33"/>
+      <c r="F28" s="33"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="34" t="s">
+        <v>64</v>
+      </c>
+      <c r="B29" s="35" t="n">
         <v>8.8</v>
       </c>
-      <c r="C28" s="28" t="s">
-        <v>62</v>
-      </c>
-      <c r="D28" s="28"/>
-      <c r="E28" s="28"/>
-    </row>
-    <row r="29" customFormat="false" ht="19.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="29" t="s">
-        <v>63</v>
-      </c>
-      <c r="B29" s="30" t="n">
+      <c r="C29" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="D29" s="33"/>
+      <c r="E29" s="33"/>
+      <c r="F29" s="33"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="34" t="s">
+        <v>66</v>
+      </c>
+      <c r="B30" s="35" t="n">
         <v>6.9</v>
       </c>
-      <c r="C29" s="28" t="s">
-        <v>64</v>
-      </c>
-      <c r="D29" s="28"/>
-      <c r="E29" s="28"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="29" t="s">
-        <v>65</v>
-      </c>
-      <c r="B30" s="30" t="n">
+      <c r="C30" s="33" t="s">
+        <v>67</v>
+      </c>
+      <c r="D30" s="33"/>
+      <c r="E30" s="33"/>
+      <c r="F30" s="33"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="34" t="s">
+        <v>68</v>
+      </c>
+      <c r="B31" s="35" t="n">
+        <v>4.33</v>
+      </c>
+      <c r="C31" s="33" t="s">
+        <v>69</v>
+      </c>
+      <c r="D31" s="33"/>
+      <c r="E31" s="33"/>
+      <c r="F31" s="33"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="34" t="s">
+        <v>70</v>
+      </c>
+      <c r="B32" s="35" t="n">
         <v>2.9</v>
       </c>
-      <c r="C30" s="28" t="s">
-        <v>66</v>
-      </c>
-      <c r="D30" s="28"/>
-      <c r="E30" s="28"/>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="29" t="s">
-        <v>67</v>
-      </c>
-      <c r="B31" s="30" t="n">
-        <v>4.33</v>
-      </c>
-      <c r="C31" s="28" t="s">
-        <v>68</v>
-      </c>
-      <c r="D31" s="28"/>
-      <c r="E31" s="28"/>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="29" t="s">
-        <v>69</v>
-      </c>
-      <c r="B32" s="30" t="n">
+      <c r="C32" s="33" t="s">
+        <v>71</v>
+      </c>
+      <c r="D32" s="33"/>
+      <c r="E32" s="33"/>
+      <c r="F32" s="33"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="34" t="s">
+        <v>72</v>
+      </c>
+      <c r="B33" s="35" t="n">
         <v>2</v>
       </c>
-      <c r="C32" s="28" t="s">
-        <v>70</v>
-      </c>
-      <c r="D32" s="28"/>
-      <c r="E32" s="28"/>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="29" t="s">
-        <v>71</v>
-      </c>
-      <c r="B33" s="30" t="n">
+      <c r="C33" s="33" t="s">
+        <v>73</v>
+      </c>
+      <c r="D33" s="33"/>
+      <c r="E33" s="33"/>
+      <c r="F33" s="33"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="34" t="s">
+        <v>74</v>
+      </c>
+      <c r="B34" s="35" t="n">
         <v>18</v>
       </c>
-      <c r="C33" s="28" t="s">
-        <v>72</v>
-      </c>
-      <c r="D33" s="28"/>
-      <c r="E33" s="28"/>
-    </row>
-    <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="31" t="s">
-        <v>73</v>
-      </c>
-      <c r="B34" s="31"/>
-      <c r="C34" s="31"/>
-      <c r="D34" s="31"/>
-      <c r="E34" s="31"/>
+      <c r="C34" s="33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D34" s="33"/>
+      <c r="E34" s="33"/>
+      <c r="F34" s="33"/>
+    </row>
+    <row r="35" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="25" t="s">
+        <v>76</v>
+      </c>
+      <c r="B35" s="25"/>
+      <c r="C35" s="25"/>
+      <c r="D35" s="25"/>
+      <c r="E35" s="25"/>
+      <c r="F35" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="C7:E7"/>
-    <mergeCell ref="A9:E9"/>
-    <mergeCell ref="A19:E19"/>
-    <mergeCell ref="A21:E21"/>
-    <mergeCell ref="C22:E22"/>
-    <mergeCell ref="C23:E23"/>
-    <mergeCell ref="C24:E24"/>
-    <mergeCell ref="C25:E25"/>
-    <mergeCell ref="C26:E26"/>
-    <mergeCell ref="C27:E27"/>
-    <mergeCell ref="C28:E28"/>
-    <mergeCell ref="C29:E29"/>
-    <mergeCell ref="C30:E30"/>
-    <mergeCell ref="C31:E31"/>
-    <mergeCell ref="C32:E32"/>
-    <mergeCell ref="C33:E33"/>
-    <mergeCell ref="A34:E34"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="C8:F8"/>
+    <mergeCell ref="A10:F10"/>
+    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A22:F22"/>
+    <mergeCell ref="C23:F23"/>
+    <mergeCell ref="C24:F24"/>
+    <mergeCell ref="C25:F25"/>
+    <mergeCell ref="C26:F26"/>
+    <mergeCell ref="C27:F27"/>
+    <mergeCell ref="C28:F28"/>
+    <mergeCell ref="C29:F29"/>
+    <mergeCell ref="C30:F30"/>
+    <mergeCell ref="C31:F31"/>
+    <mergeCell ref="C32:F32"/>
+    <mergeCell ref="C33:F33"/>
+    <mergeCell ref="C34:F34"/>
+    <mergeCell ref="A35:F35"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2591,7 +2647,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2600,7 +2656,7 @@
     </row>
     <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -2609,7 +2665,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B4" s="14"/>
       <c r="C4" s="14"/>
@@ -2618,155 +2674,155 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="B5" s="32" t="n">
+        <v>80</v>
+      </c>
+      <c r="B5" s="36" t="n">
         <v>631805</v>
       </c>
-      <c r="E5" s="33" t="s">
-        <v>78</v>
+      <c r="E5" s="37" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="B6" s="34" t="n">
+        <v>82</v>
+      </c>
+      <c r="B6" s="38" t="n">
         <v>0.5</v>
       </c>
-      <c r="E6" s="33" t="s">
-        <v>80</v>
+      <c r="E6" s="37" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="B7" s="34" t="n">
+        <v>84</v>
+      </c>
+      <c r="B7" s="38" t="n">
         <v>0.73</v>
       </c>
-      <c r="E7" s="33" t="s">
-        <v>82</v>
+      <c r="E7" s="37" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="B8" s="24" t="n">
+        <v>86</v>
+      </c>
+      <c r="B8" s="22" t="n">
         <f aca="false">Australia!B18</f>
         <v>0.3</v>
       </c>
-      <c r="E8" s="33" t="s">
-        <v>84</v>
+      <c r="E8" s="37" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="B9" s="34" t="n">
+        <v>88</v>
+      </c>
+      <c r="B9" s="38" t="n">
         <v>0.51</v>
       </c>
-      <c r="E9" s="33" t="s">
-        <v>86</v>
+      <c r="E9" s="37" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="B10" s="35" t="n">
+        <v>90</v>
+      </c>
+      <c r="B10" s="39" t="n">
         <f aca="false">Australia!B25</f>
         <v>2.29828645030564</v>
       </c>
-      <c r="E10" s="33" t="s">
-        <v>88</v>
+      <c r="E10" s="37" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="B11" s="36" t="n">
+        <v>92</v>
+      </c>
+      <c r="B11" s="40" t="n">
         <f aca="false">1-B8</f>
         <v>0.7</v>
       </c>
-      <c r="E11" s="33" t="s">
-        <v>90</v>
+      <c r="E11" s="37" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="B12" s="37" t="n">
+        <v>94</v>
+      </c>
+      <c r="B12" s="41" t="n">
         <v>600</v>
       </c>
-      <c r="E12" s="33" t="s">
-        <v>92</v>
+      <c r="E12" s="37" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="B13" s="34" t="n">
+        <v>96</v>
+      </c>
+      <c r="B13" s="38" t="n">
         <v>0.075</v>
       </c>
-      <c r="E13" s="33" t="s">
-        <v>94</v>
+      <c r="E13" s="37" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="B14" s="32" t="n">
+        <v>98</v>
+      </c>
+      <c r="B14" s="36" t="n">
         <v>3</v>
       </c>
-      <c r="E14" s="33" t="s">
-        <v>96</v>
+      <c r="E14" s="37" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="B15" s="32" t="n">
+        <v>100</v>
+      </c>
+      <c r="B15" s="36" t="n">
         <v>87000</v>
       </c>
-      <c r="E15" s="33" t="s">
-        <v>98</v>
+      <c r="E15" s="37" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="B16" s="34" t="n">
+        <v>102</v>
+      </c>
+      <c r="B16" s="38" t="n">
         <v>0.4</v>
       </c>
-      <c r="E16" s="33" t="s">
-        <v>100</v>
+      <c r="E16" s="37" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="17"/>
-      <c r="B18" s="38" t="s">
-        <v>101</v>
-      </c>
-      <c r="C18" s="38" t="s">
-        <v>34</v>
-      </c>
-      <c r="D18" s="38" t="s">
-        <v>102</v>
-      </c>
-      <c r="E18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="43" t="s">
+        <v>104</v>
+      </c>
+      <c r="C18" s="43" t="s">
+        <v>105</v>
+      </c>
+      <c r="D18" s="43" t="s">
+        <v>106</v>
+      </c>
+      <c r="E18" s="44"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="14" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B19" s="14"/>
       <c r="C19" s="14"/>
@@ -2774,25 +2830,25 @@
       <c r="E19" s="14"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="40" t="s">
-        <v>104</v>
-      </c>
-      <c r="B20" s="41" t="n">
+      <c r="A20" s="45" t="s">
+        <v>108</v>
+      </c>
+      <c r="B20" s="46" t="n">
         <f aca="false">$B$5*$B$6</f>
         <v>315902.5</v>
       </c>
-      <c r="C20" s="41" t="n">
+      <c r="C20" s="46" t="n">
         <f aca="false">$B$5*$B$7</f>
         <v>461217.65</v>
       </c>
-      <c r="D20" s="41" t="n">
+      <c r="D20" s="46" t="n">
         <f aca="false">$B$5</f>
         <v>631805</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="42" t="s">
-        <v>105</v>
+      <c r="A21" s="47" t="s">
+        <v>109</v>
       </c>
       <c r="B21" s="10" t="n">
         <f aca="false">B20*$B$8</f>
@@ -2808,8 +2864,8 @@
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="42" t="s">
-        <v>106</v>
+      <c r="A22" s="47" t="s">
+        <v>110</v>
       </c>
       <c r="B22" s="10" t="n">
         <f aca="false">B20*$B$11</f>
@@ -2826,7 +2882,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="14" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="B23" s="14"/>
       <c r="C23" s="14"/>
@@ -2834,79 +2890,79 @@
       <c r="E23" s="14"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="40" t="s">
-        <v>108</v>
-      </c>
-      <c r="B24" s="43" t="n">
+      <c r="A24" s="45" t="s">
+        <v>112</v>
+      </c>
+      <c r="B24" s="48" t="n">
         <f aca="false">B20*$B$9*$B$8/$B$10</f>
         <v>21030.0515384287</v>
       </c>
-      <c r="C24" s="43" t="n">
+      <c r="C24" s="48" t="n">
         <f aca="false">C20*$B$9*$B$8/$B$10</f>
         <v>30703.875246106</v>
       </c>
-      <c r="D24" s="43" t="n">
+      <c r="D24" s="48" t="n">
         <f aca="false">D20*$B$9*$B$8/$B$10</f>
         <v>42060.1030768575</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="40" t="s">
-        <v>109</v>
-      </c>
-      <c r="B25" s="41" t="n">
+      <c r="A25" s="45" t="s">
+        <v>113</v>
+      </c>
+      <c r="B25" s="46" t="n">
         <f aca="false">B20*$B$9*$B$8</f>
         <v>48333.0825</v>
       </c>
-      <c r="C25" s="41" t="n">
+      <c r="C25" s="46" t="n">
         <f aca="false">C20*$B$9*$B$8</f>
         <v>70566.30045</v>
       </c>
-      <c r="D25" s="41" t="n">
+      <c r="D25" s="46" t="n">
         <f aca="false">D20*$B$9*$B$8</f>
         <v>96666.165</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="42" t="s">
-        <v>110</v>
-      </c>
-      <c r="B26" s="44" t="n">
+      <c r="A26" s="47" t="s">
+        <v>114</v>
+      </c>
+      <c r="B26" s="49" t="n">
         <f aca="false">B25*Summary!$B$5</f>
         <v>24166.54125</v>
       </c>
-      <c r="C26" s="44" t="n">
+      <c r="C26" s="49" t="n">
         <f aca="false">C25*Summary!$B$5</f>
         <v>35283.150225</v>
       </c>
-      <c r="D26" s="44" t="n">
+      <c r="D26" s="49" t="n">
         <f aca="false">D25*Summary!$B$5</f>
         <v>48333.0825</v>
       </c>
-      <c r="E26" s="33" t="s">
-        <v>111</v>
+      <c r="E26" s="37" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="42" t="s">
-        <v>112</v>
-      </c>
-      <c r="B27" s="32" t="n">
+      <c r="A27" s="47" t="s">
+        <v>116</v>
+      </c>
+      <c r="B27" s="36" t="n">
         <v>1120</v>
       </c>
-      <c r="C27" s="32" t="n">
+      <c r="C27" s="36" t="n">
         <v>1540</v>
       </c>
-      <c r="D27" s="32" t="n">
+      <c r="D27" s="36" t="n">
         <v>2110</v>
       </c>
-      <c r="E27" s="33" t="s">
-        <v>113</v>
+      <c r="E27" s="37" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="14" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="B28" s="14"/>
       <c r="C28" s="14"/>
@@ -2914,48 +2970,48 @@
       <c r="E28" s="14"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="42" t="s">
-        <v>115</v>
-      </c>
-      <c r="B29" s="45" t="n">
+      <c r="A29" s="47" t="s">
+        <v>119</v>
+      </c>
+      <c r="B29" s="50" t="n">
         <f aca="false">B20*$B$14</f>
         <v>947707.5</v>
       </c>
-      <c r="C29" s="45" t="n">
+      <c r="C29" s="50" t="n">
         <f aca="false">C20*$B$14</f>
         <v>1383652.95</v>
       </c>
-      <c r="D29" s="45" t="n">
+      <c r="D29" s="50" t="n">
         <f aca="false">D20*$B$14</f>
         <v>1895415</v>
       </c>
-      <c r="E29" s="33" t="s">
-        <v>116</v>
+      <c r="E29" s="37" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="40" t="s">
-        <v>117</v>
-      </c>
-      <c r="B30" s="46" t="n">
+      <c r="A30" s="45" t="s">
+        <v>121</v>
+      </c>
+      <c r="B30" s="51" t="n">
         <f aca="false">B20*$B$12*52*$B$13</f>
         <v>739211850</v>
       </c>
-      <c r="C30" s="46" t="n">
+      <c r="C30" s="51" t="n">
         <f aca="false">C20*$B$12*52*$B$13</f>
         <v>1079249301</v>
       </c>
-      <c r="D30" s="46" t="n">
+      <c r="D30" s="51" t="n">
         <f aca="false">D20*$B$12*52*$B$13</f>
         <v>1478423700</v>
       </c>
-      <c r="E30" s="33" t="s">
-        <v>118</v>
+      <c r="E30" s="37" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="42" t="s">
-        <v>119</v>
+      <c r="A31" s="47" t="s">
+        <v>123</v>
       </c>
       <c r="B31" s="10" t="n">
         <f aca="false">$B$15*$B$6</f>
@@ -2971,48 +3027,48 @@
       </c>
     </row>
     <row r="32" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="42" t="s">
-        <v>120</v>
-      </c>
-      <c r="B32" s="45" t="n">
+      <c r="A32" s="47" t="s">
+        <v>124</v>
+      </c>
+      <c r="B32" s="50" t="n">
         <f aca="false">B31*$B$16</f>
         <v>17400</v>
       </c>
-      <c r="C32" s="45" t="n">
+      <c r="C32" s="50" t="n">
         <f aca="false">C31*$B$16</f>
         <v>25404</v>
       </c>
-      <c r="D32" s="45" t="n">
+      <c r="D32" s="50" t="n">
         <f aca="false">D31*$B$16</f>
         <v>34800</v>
       </c>
-      <c r="E32" s="33" t="s">
-        <v>121</v>
+      <c r="E32" s="37" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="40" t="s">
-        <v>122</v>
-      </c>
-      <c r="B33" s="47" t="n">
+      <c r="A33" s="45" t="s">
+        <v>126</v>
+      </c>
+      <c r="B33" s="52" t="n">
         <f aca="false">B26*$B$14</f>
         <v>72499.62375</v>
       </c>
-      <c r="C33" s="47" t="n">
+      <c r="C33" s="52" t="n">
         <f aca="false">C26*$B$14</f>
         <v>105849.450675</v>
       </c>
-      <c r="D33" s="47" t="n">
+      <c r="D33" s="52" t="n">
         <f aca="false">D26*$B$14</f>
         <v>144999.2475</v>
       </c>
-      <c r="E33" s="33" t="s">
-        <v>123</v>
+      <c r="E33" s="37" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="14" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B35" s="14"/>
       <c r="C35" s="14"/>
@@ -3020,58 +3076,58 @@
       <c r="E35" s="14"/>
     </row>
     <row r="36" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="48" t="s">
-        <v>125</v>
-      </c>
-      <c r="B36" s="48"/>
-      <c r="C36" s="48"/>
-      <c r="D36" s="48"/>
-      <c r="E36" s="48"/>
+      <c r="A36" s="53" t="s">
+        <v>129</v>
+      </c>
+      <c r="B36" s="53"/>
+      <c r="C36" s="53"/>
+      <c r="D36" s="53"/>
+      <c r="E36" s="53"/>
     </row>
     <row r="37" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="48" t="s">
-        <v>126</v>
-      </c>
-      <c r="B37" s="48"/>
-      <c r="C37" s="48"/>
-      <c r="D37" s="48"/>
-      <c r="E37" s="48"/>
+      <c r="A37" s="53" t="s">
+        <v>130</v>
+      </c>
+      <c r="B37" s="53"/>
+      <c r="C37" s="53"/>
+      <c r="D37" s="53"/>
+      <c r="E37" s="53"/>
     </row>
     <row r="38" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="48" t="s">
-        <v>127</v>
-      </c>
-      <c r="B38" s="48"/>
-      <c r="C38" s="48"/>
-      <c r="D38" s="48"/>
-      <c r="E38" s="48"/>
+      <c r="A38" s="53" t="s">
+        <v>131</v>
+      </c>
+      <c r="B38" s="53"/>
+      <c r="C38" s="53"/>
+      <c r="D38" s="53"/>
+      <c r="E38" s="53"/>
     </row>
     <row r="39" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="48" t="s">
-        <v>128</v>
-      </c>
-      <c r="B39" s="48"/>
-      <c r="C39" s="48"/>
-      <c r="D39" s="48"/>
-      <c r="E39" s="48"/>
+      <c r="A39" s="53" t="s">
+        <v>132</v>
+      </c>
+      <c r="B39" s="53"/>
+      <c r="C39" s="53"/>
+      <c r="D39" s="53"/>
+      <c r="E39" s="53"/>
     </row>
     <row r="40" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="48" t="s">
-        <v>129</v>
-      </c>
-      <c r="B40" s="48"/>
-      <c r="C40" s="48"/>
-      <c r="D40" s="48"/>
-      <c r="E40" s="48"/>
+      <c r="A40" s="53" t="s">
+        <v>133</v>
+      </c>
+      <c r="B40" s="53"/>
+      <c r="C40" s="53"/>
+      <c r="D40" s="53"/>
+      <c r="E40" s="53"/>
     </row>
     <row r="42" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="49" t="s">
-        <v>130</v>
-      </c>
-      <c r="B42" s="49"/>
-      <c r="C42" s="49"/>
-      <c r="D42" s="49"/>
-      <c r="E42" s="49"/>
+      <c r="A42" s="54" t="s">
+        <v>134</v>
+      </c>
+      <c r="B42" s="54"/>
+      <c r="C42" s="54"/>
+      <c r="D42" s="54"/>
+      <c r="E42" s="54"/>
     </row>
   </sheetData>
   <mergeCells count="13">
@@ -3117,7 +3173,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3126,18 +3182,18 @@
       <c r="F1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="50" t="s">
-        <v>132</v>
-      </c>
-      <c r="B2" s="50"/>
-      <c r="C2" s="50"/>
-      <c r="D2" s="50"/>
-      <c r="E2" s="50"/>
-      <c r="F2" s="50"/>
+      <c r="A2" s="55" t="s">
+        <v>136</v>
+      </c>
+      <c r="B2" s="55"/>
+      <c r="C2" s="55"/>
+      <c r="D2" s="55"/>
+      <c r="E2" s="55"/>
+      <c r="F2" s="55"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="B4" s="14"/>
       <c r="C4" s="14"/>
@@ -3147,126 +3203,126 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5"/>
-      <c r="B5" s="51" t="s">
-        <v>134</v>
-      </c>
-      <c r="C5" s="52" t="s">
-        <v>135</v>
+      <c r="B5" s="56" t="s">
+        <v>138</v>
+      </c>
+      <c r="C5" s="57" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="40" t="s">
-        <v>136</v>
-      </c>
-      <c r="B6" s="53" t="s">
-        <v>137</v>
-      </c>
-      <c r="C6" s="54" t="s">
-        <v>138</v>
+      <c r="A6" s="45" t="s">
+        <v>140</v>
+      </c>
+      <c r="B6" s="58" t="s">
+        <v>141</v>
+      </c>
+      <c r="C6" s="59" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="40" t="s">
-        <v>139</v>
-      </c>
-      <c r="B7" s="53" t="s">
-        <v>140</v>
-      </c>
-      <c r="C7" s="54" t="s">
-        <v>141</v>
+      <c r="A7" s="45" t="s">
+        <v>143</v>
+      </c>
+      <c r="B7" s="58" t="s">
+        <v>144</v>
+      </c>
+      <c r="C7" s="59" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="40" t="s">
-        <v>142</v>
-      </c>
-      <c r="B8" s="53" t="s">
-        <v>143</v>
-      </c>
-      <c r="C8" s="54" t="s">
-        <v>144</v>
+      <c r="A8" s="45" t="s">
+        <v>146</v>
+      </c>
+      <c r="B8" s="58" t="s">
+        <v>147</v>
+      </c>
+      <c r="C8" s="59" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="40" t="s">
-        <v>145</v>
-      </c>
-      <c r="B9" s="53" t="s">
-        <v>146</v>
-      </c>
-      <c r="C9" s="54" t="s">
-        <v>147</v>
+      <c r="A9" s="45" t="s">
+        <v>149</v>
+      </c>
+      <c r="B9" s="58" t="s">
+        <v>150</v>
+      </c>
+      <c r="C9" s="59" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="40" t="s">
-        <v>148</v>
-      </c>
-      <c r="B10" s="53" t="s">
-        <v>149</v>
-      </c>
-      <c r="C10" s="54" t="s">
-        <v>150</v>
+      <c r="A10" s="45" t="s">
+        <v>152</v>
+      </c>
+      <c r="B10" s="58" t="s">
+        <v>153</v>
+      </c>
+      <c r="C10" s="59" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="40" t="s">
-        <v>151</v>
-      </c>
-      <c r="B11" s="53" t="s">
-        <v>152</v>
-      </c>
-      <c r="C11" s="54" t="s">
-        <v>153</v>
+      <c r="A11" s="45" t="s">
+        <v>155</v>
+      </c>
+      <c r="B11" s="58" t="s">
+        <v>156</v>
+      </c>
+      <c r="C11" s="59" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="40" t="s">
-        <v>154</v>
-      </c>
-      <c r="B12" s="53" t="s">
-        <v>155</v>
-      </c>
-      <c r="C12" s="54" t="s">
-        <v>156</v>
+      <c r="A12" s="45" t="s">
+        <v>158</v>
+      </c>
+      <c r="B12" s="58" t="s">
+        <v>159</v>
+      </c>
+      <c r="C12" s="59" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="40" t="s">
-        <v>157</v>
-      </c>
-      <c r="B13" s="53" t="s">
-        <v>158</v>
-      </c>
-      <c r="C13" s="54" t="s">
-        <v>159</v>
+      <c r="A13" s="45" t="s">
+        <v>161</v>
+      </c>
+      <c r="B13" s="58" t="s">
+        <v>162</v>
+      </c>
+      <c r="C13" s="59" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="40" t="s">
-        <v>160</v>
-      </c>
-      <c r="B14" s="53" t="s">
-        <v>161</v>
-      </c>
-      <c r="C14" s="54" t="s">
-        <v>162</v>
+      <c r="A14" s="45" t="s">
+        <v>164</v>
+      </c>
+      <c r="B14" s="58" t="s">
+        <v>165</v>
+      </c>
+      <c r="C14" s="59" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="40" t="s">
-        <v>163</v>
-      </c>
-      <c r="B15" s="53" t="s">
-        <v>164</v>
-      </c>
-      <c r="C15" s="54" t="s">
-        <v>165</v>
+      <c r="A15" s="45" t="s">
+        <v>167</v>
+      </c>
+      <c r="B15" s="58" t="s">
+        <v>168</v>
+      </c>
+      <c r="C15" s="59" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="B17" s="14"/>
       <c r="C17" s="14"/>
@@ -3276,14 +3332,14 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="B18" s="55" t="n">
+        <v>171</v>
+      </c>
+      <c r="B18" s="60" t="n">
         <f aca="false">Summary!B6</f>
         <v>3</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="D18" s="3"/>
       <c r="E18" s="3"/>
@@ -3291,13 +3347,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="B19" s="7" t="n">
         <v>3.5</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="D19" s="3"/>
       <c r="E19" s="3"/>
@@ -3305,13 +3361,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>171</v>
-      </c>
-      <c r="B20" s="56" t="n">
+        <v>175</v>
+      </c>
+      <c r="B20" s="61" t="n">
         <v>150</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="D20" s="3"/>
       <c r="E20" s="3"/>
@@ -3319,13 +3375,13 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>173</v>
-      </c>
-      <c r="B21" s="56" t="n">
+        <v>177</v>
+      </c>
+      <c r="B21" s="61" t="n">
         <v>2500</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="D21" s="3"/>
       <c r="E21" s="3"/>
@@ -3333,13 +3389,13 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>175</v>
-      </c>
-      <c r="B22" s="56" t="n">
+        <v>179</v>
+      </c>
+      <c r="B22" s="61" t="n">
         <v>0</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="D22" s="3"/>
       <c r="E22" s="3"/>
@@ -3347,7 +3403,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="14" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="B24" s="14"/>
       <c r="C24" s="14"/>
@@ -3356,171 +3412,171 @@
       <c r="F24" s="14"/>
     </row>
     <row r="25" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="38" t="s">
-        <v>178</v>
-      </c>
-      <c r="B25" s="38" t="s">
-        <v>179</v>
-      </c>
-      <c r="C25" s="38" t="s">
-        <v>180</v>
-      </c>
-      <c r="D25" s="38" t="s">
-        <v>181</v>
-      </c>
-      <c r="E25" s="38" t="s">
+      <c r="A25" s="43" t="s">
         <v>182</v>
       </c>
-      <c r="F25" s="38" t="s">
+      <c r="B25" s="43" t="s">
         <v>183</v>
       </c>
+      <c r="C25" s="43" t="s">
+        <v>184</v>
+      </c>
+      <c r="D25" s="43" t="s">
+        <v>185</v>
+      </c>
+      <c r="E25" s="43" t="s">
+        <v>186</v>
+      </c>
+      <c r="F25" s="43" t="s">
+        <v>187</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="57" t="n">
+      <c r="A26" s="62" t="n">
         <v>5</v>
       </c>
-      <c r="B26" s="58" t="n">
+      <c r="B26" s="63" t="n">
         <f aca="false">A26*$B$18*12</f>
         <v>180</v>
       </c>
-      <c r="C26" s="59" t="n">
+      <c r="C26" s="64" t="n">
         <f aca="false">MAX(A26*$B$19,$B$20)*12</f>
         <v>1800</v>
       </c>
-      <c r="D26" s="59" t="n">
+      <c r="D26" s="64" t="n">
         <f aca="false">C26+$B$21</f>
         <v>4300</v>
       </c>
-      <c r="E26" s="60" t="n">
+      <c r="E26" s="65" t="n">
         <f aca="false">B26/A26/12</f>
         <v>3</v>
       </c>
-      <c r="F26" s="60" t="n">
+      <c r="F26" s="65" t="n">
         <f aca="false">D26/A26/12</f>
         <v>71.6666666666667</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="57" t="n">
+      <c r="A27" s="62" t="n">
         <v>10</v>
       </c>
-      <c r="B27" s="58" t="n">
+      <c r="B27" s="63" t="n">
         <f aca="false">A27*$B$18*12</f>
         <v>360</v>
       </c>
-      <c r="C27" s="59" t="n">
+      <c r="C27" s="64" t="n">
         <f aca="false">MAX(A27*$B$19,$B$20)*12</f>
         <v>1800</v>
       </c>
-      <c r="D27" s="59" t="n">
+      <c r="D27" s="64" t="n">
         <f aca="false">C27+$B$21</f>
         <v>4300</v>
       </c>
-      <c r="E27" s="60" t="n">
+      <c r="E27" s="65" t="n">
         <f aca="false">B27/A27/12</f>
         <v>3</v>
       </c>
-      <c r="F27" s="60" t="n">
+      <c r="F27" s="65" t="n">
         <f aca="false">D27/A27/12</f>
         <v>35.8333333333333</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="57" t="n">
+      <c r="A28" s="62" t="n">
         <v>20</v>
       </c>
-      <c r="B28" s="58" t="n">
+      <c r="B28" s="63" t="n">
         <f aca="false">A28*$B$18*12</f>
         <v>720</v>
       </c>
-      <c r="C28" s="59" t="n">
+      <c r="C28" s="64" t="n">
         <f aca="false">MAX(A28*$B$19,$B$20)*12</f>
         <v>1800</v>
       </c>
-      <c r="D28" s="59" t="n">
+      <c r="D28" s="64" t="n">
         <f aca="false">C28+$B$21</f>
         <v>4300</v>
       </c>
-      <c r="E28" s="60" t="n">
+      <c r="E28" s="65" t="n">
         <f aca="false">B28/A28/12</f>
         <v>3</v>
       </c>
-      <c r="F28" s="60" t="n">
+      <c r="F28" s="65" t="n">
         <f aca="false">D28/A28/12</f>
         <v>17.9166666666667</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="57" t="n">
+      <c r="A29" s="62" t="n">
         <v>50</v>
       </c>
-      <c r="B29" s="58" t="n">
+      <c r="B29" s="63" t="n">
         <f aca="false">A29*$B$18*12</f>
         <v>1800</v>
       </c>
-      <c r="C29" s="59" t="n">
+      <c r="C29" s="64" t="n">
         <f aca="false">MAX(A29*$B$19,$B$20)*12</f>
         <v>2100</v>
       </c>
-      <c r="D29" s="59" t="n">
+      <c r="D29" s="64" t="n">
         <f aca="false">C29+$B$21</f>
         <v>4600</v>
       </c>
-      <c r="E29" s="60" t="n">
+      <c r="E29" s="65" t="n">
         <f aca="false">B29/A29/12</f>
         <v>3</v>
       </c>
-      <c r="F29" s="60" t="n">
+      <c r="F29" s="65" t="n">
         <f aca="false">D29/A29/12</f>
         <v>7.66666666666667</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="57" t="n">
+      <c r="A30" s="62" t="n">
         <v>100</v>
       </c>
-      <c r="B30" s="58" t="n">
+      <c r="B30" s="63" t="n">
         <f aca="false">A30*$B$18*12</f>
         <v>3600</v>
       </c>
-      <c r="C30" s="59" t="n">
+      <c r="C30" s="64" t="n">
         <f aca="false">MAX(A30*$B$19,$B$20)*12</f>
         <v>4200</v>
       </c>
-      <c r="D30" s="59" t="n">
+      <c r="D30" s="64" t="n">
         <f aca="false">C30+$B$21</f>
         <v>6700</v>
       </c>
-      <c r="E30" s="60" t="n">
+      <c r="E30" s="65" t="n">
         <f aca="false">B30/A30/12</f>
         <v>3</v>
       </c>
-      <c r="F30" s="60" t="n">
+      <c r="F30" s="65" t="n">
         <f aca="false">D30/A30/12</f>
         <v>5.58333333333333</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="31" t="s">
-        <v>184</v>
-      </c>
-      <c r="B31" s="31"/>
-      <c r="C31" s="31"/>
-      <c r="D31" s="31"/>
-      <c r="E31" s="31"/>
-      <c r="F31" s="31"/>
+      <c r="A31" s="25" t="s">
+        <v>188</v>
+      </c>
+      <c r="B31" s="25"/>
+      <c r="C31" s="25"/>
+      <c r="D31" s="25"/>
+      <c r="E31" s="25"/>
+      <c r="F31" s="25"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="31"/>
-      <c r="B32" s="31"/>
-      <c r="C32" s="31"/>
-      <c r="D32" s="31"/>
-      <c r="E32" s="31"/>
-      <c r="F32" s="31"/>
+      <c r="A32" s="25"/>
+      <c r="B32" s="25"/>
+      <c r="C32" s="25"/>
+      <c r="D32" s="25"/>
+      <c r="E32" s="25"/>
+      <c r="F32" s="25"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="14" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="B34" s="14"/>
       <c r="C34" s="14"/>
@@ -3529,54 +3585,54 @@
       <c r="F34" s="14"/>
     </row>
     <row r="35" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="48" t="s">
-        <v>186</v>
-      </c>
-      <c r="B35" s="48"/>
-      <c r="C35" s="48"/>
-      <c r="D35" s="48"/>
-      <c r="E35" s="48"/>
-      <c r="F35" s="48"/>
+      <c r="A35" s="53" t="s">
+        <v>190</v>
+      </c>
+      <c r="B35" s="53"/>
+      <c r="C35" s="53"/>
+      <c r="D35" s="53"/>
+      <c r="E35" s="53"/>
+      <c r="F35" s="53"/>
     </row>
     <row r="36" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="48" t="s">
-        <v>187</v>
-      </c>
-      <c r="B36" s="48"/>
-      <c r="C36" s="48"/>
-      <c r="D36" s="48"/>
-      <c r="E36" s="48"/>
-      <c r="F36" s="48"/>
+      <c r="A36" s="53" t="s">
+        <v>191</v>
+      </c>
+      <c r="B36" s="53"/>
+      <c r="C36" s="53"/>
+      <c r="D36" s="53"/>
+      <c r="E36" s="53"/>
+      <c r="F36" s="53"/>
     </row>
     <row r="37" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="48" t="s">
-        <v>188</v>
-      </c>
-      <c r="B37" s="48"/>
-      <c r="C37" s="48"/>
-      <c r="D37" s="48"/>
-      <c r="E37" s="48"/>
-      <c r="F37" s="48"/>
+      <c r="A37" s="53" t="s">
+        <v>192</v>
+      </c>
+      <c r="B37" s="53"/>
+      <c r="C37" s="53"/>
+      <c r="D37" s="53"/>
+      <c r="E37" s="53"/>
+      <c r="F37" s="53"/>
     </row>
     <row r="38" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="48" t="s">
-        <v>189</v>
-      </c>
-      <c r="B38" s="48"/>
-      <c r="C38" s="48"/>
-      <c r="D38" s="48"/>
-      <c r="E38" s="48"/>
-      <c r="F38" s="48"/>
+      <c r="A38" s="53" t="s">
+        <v>193</v>
+      </c>
+      <c r="B38" s="53"/>
+      <c r="C38" s="53"/>
+      <c r="D38" s="53"/>
+      <c r="E38" s="53"/>
+      <c r="F38" s="53"/>
     </row>
     <row r="39" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="48" t="s">
-        <v>190</v>
-      </c>
-      <c r="B39" s="48"/>
-      <c r="C39" s="48"/>
-      <c r="D39" s="48"/>
-      <c r="E39" s="48"/>
-      <c r="F39" s="48"/>
+      <c r="A39" s="53" t="s">
+        <v>194</v>
+      </c>
+      <c r="B39" s="53"/>
+      <c r="C39" s="53"/>
+      <c r="D39" s="53"/>
+      <c r="E39" s="53"/>
+      <c r="F39" s="53"/>
     </row>
   </sheetData>
   <mergeCells count="17">
@@ -3624,88 +3680,88 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="61" t="s">
-        <v>191</v>
-      </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
+      <c r="A1" s="66" t="s">
+        <v>195</v>
+      </c>
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="B3" s="14"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>193</v>
-      </c>
-      <c r="B4" s="62" t="n">
+        <v>197</v>
+      </c>
+      <c r="B4" s="67" t="n">
         <v>1620633</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>194</v>
-      </c>
-      <c r="B5" s="62" t="n">
+        <v>198</v>
+      </c>
+      <c r="B5" s="67" t="n">
         <v>428020</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>195</v>
-      </c>
-      <c r="B6" s="62" t="n">
+        <v>199</v>
+      </c>
+      <c r="B6" s="67" t="n">
         <v>132338</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>196</v>
-      </c>
-      <c r="B7" s="62" t="n">
+        <v>200</v>
+      </c>
+      <c r="B7" s="67" t="n">
         <v>47633</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>197</v>
-      </c>
-      <c r="B8" s="62" t="n">
+        <v>201</v>
+      </c>
+      <c r="B8" s="67" t="n">
         <v>19530</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>198</v>
-      </c>
-      <c r="B9" s="62" t="n">
+        <v>202</v>
+      </c>
+      <c r="B9" s="67" t="n">
         <v>19977</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="19" t="s">
-        <v>199</v>
-      </c>
-      <c r="B10" s="43" t="n">
+      <c r="A10" s="23" t="s">
+        <v>203</v>
+      </c>
+      <c r="B10" s="48" t="n">
         <f aca="false">SUM(B4:B9)</f>
         <v>2268131</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="19" t="s">
-        <v>200</v>
-      </c>
-      <c r="B11" s="43" t="n">
+      <c r="A11" s="23" t="s">
+        <v>204</v>
+      </c>
+      <c r="B11" s="48" t="n">
         <f aca="false">SUM(B5:B9)</f>
         <v>647498</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="B12" s="10" t="n">
         <f aca="false">B4</f>
@@ -3714,86 +3770,86 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="B14" s="14"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>203</v>
-      </c>
-      <c r="B15" s="63" t="n">
+        <v>207</v>
+      </c>
+      <c r="B15" s="68" t="n">
         <v>7.5</v>
       </c>
-      <c r="D15" s="33" t="s">
-        <v>204</v>
+      <c r="D15" s="37" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>205</v>
-      </c>
-      <c r="B16" s="63" t="n">
+        <v>209</v>
+      </c>
+      <c r="B16" s="68" t="n">
         <v>0.88</v>
       </c>
-      <c r="D16" s="33" t="s">
-        <v>206</v>
+      <c r="D16" s="37" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>207</v>
-      </c>
-      <c r="B17" s="32" t="n">
+        <v>211</v>
+      </c>
+      <c r="B17" s="36" t="n">
         <v>2900000</v>
       </c>
-      <c r="D17" s="33" t="s">
-        <v>208</v>
+      <c r="D17" s="37" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="B18" s="34" t="n">
+        <v>86</v>
+      </c>
+      <c r="B18" s="38" t="n">
         <v>0.3</v>
       </c>
-      <c r="D18" s="33" t="s">
-        <v>209</v>
+      <c r="D18" s="37" t="s">
+        <v>213</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="B19" s="36" t="n">
+        <v>92</v>
+      </c>
+      <c r="B19" s="40" t="n">
         <f aca="false">1-B18</f>
         <v>0.7</v>
       </c>
-      <c r="D19" s="33" t="s">
-        <v>90</v>
+      <c r="D19" s="37" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>210</v>
-      </c>
-      <c r="B20" s="32" t="n">
+        <v>214</v>
+      </c>
+      <c r="B20" s="36" t="n">
         <v>11784</v>
       </c>
-      <c r="D20" s="33" t="s">
-        <v>211</v>
+      <c r="D20" s="37" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="14" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="B22" s="14"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="B23" s="10" t="n">
         <f aca="false">B5*2+B6*3+B7*4+B8*5+B9*B15</f>
@@ -3802,7 +3858,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="B24" s="10" t="n">
         <f aca="false">B23*B16</f>
@@ -3811,40 +3867,40 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>215</v>
-      </c>
-      <c r="B25" s="64" t="n">
+        <v>219</v>
+      </c>
+      <c r="B25" s="69" t="n">
         <f aca="false">B24/B11</f>
         <v>2.29828645030564</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="14" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="B26" s="14"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="19" t="s">
-        <v>217</v>
-      </c>
-      <c r="B27" s="43" t="n">
+      <c r="A27" s="23" t="s">
+        <v>221</v>
+      </c>
+      <c r="B27" s="48" t="n">
         <f aca="false">B11*B18</f>
         <v>194249.4</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="19" t="s">
-        <v>218</v>
-      </c>
-      <c r="B28" s="43" t="n">
+      <c r="A28" s="23" t="s">
+        <v>222</v>
+      </c>
+      <c r="B28" s="48" t="n">
         <f aca="false">B24*B18</f>
         <v>446440.764</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="B29" s="9" t="n">
         <f aca="false">B27*Summary!B5</f>
@@ -3853,7 +3909,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="B30" s="9" t="n">
         <f aca="false">B28*Summary!B5</f>
@@ -3862,31 +3918,31 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="14" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="B32" s="14"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="19" t="s">
-        <v>222</v>
-      </c>
-      <c r="B33" s="43" t="n">
+      <c r="A33" s="23" t="s">
+        <v>226</v>
+      </c>
+      <c r="B33" s="48" t="n">
         <f aca="false">B20</f>
         <v>11784</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="19" t="s">
-        <v>223</v>
-      </c>
-      <c r="B34" s="43" t="n">
+      <c r="A34" s="23" t="s">
+        <v>227</v>
+      </c>
+      <c r="B34" s="48" t="n">
         <f aca="false">B17*B19</f>
         <v>2030000</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="B35" s="10" t="n">
         <f aca="false">B34/B20</f>
@@ -3895,7 +3951,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="B36" s="9" t="n">
         <f aca="false">B33*Summary!B5</f>
@@ -3904,7 +3960,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="B37" s="9" t="n">
         <f aca="false">B34*Summary!B5</f>
@@ -3913,17 +3969,17 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="16" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="B39" s="16"/>
       <c r="C39" s="16"/>
       <c r="D39" s="16"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="65" t="s">
-        <v>227</v>
-      </c>
-      <c r="B40" s="66" t="n">
+      <c r="A40" s="70" t="s">
+        <v>231</v>
+      </c>
+      <c r="B40" s="71" t="n">
         <f aca="false">B12*B16*B18</f>
         <v>427847.112</v>
       </c>
@@ -3964,104 +4020,104 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="61" t="s">
-        <v>228</v>
-      </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
+      <c r="A1" s="66" t="s">
+        <v>232</v>
+      </c>
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="B3" s="14"/>
     </row>
     <row r="4" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>230</v>
-      </c>
-      <c r="B4" s="32" t="n">
+        <v>234</v>
+      </c>
+      <c r="B4" s="36" t="n">
         <v>600000</v>
       </c>
-      <c r="D4" s="33" t="s">
-        <v>231</v>
+      <c r="D4" s="37" t="s">
+        <v>235</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>232</v>
-      </c>
-      <c r="B5" s="34" t="n">
+        <v>236</v>
+      </c>
+      <c r="B5" s="38" t="n">
         <v>0.8</v>
       </c>
-      <c r="D5" s="33" t="s">
-        <v>233</v>
+      <c r="D5" s="37" t="s">
+        <v>237</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="B6" s="34" t="n">
+        <v>238</v>
+      </c>
+      <c r="B6" s="38" t="n">
         <v>0.5</v>
       </c>
-      <c r="D6" s="33" t="s">
-        <v>235</v>
+      <c r="D6" s="37" t="s">
+        <v>239</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="B7" s="34" t="n">
+        <v>86</v>
+      </c>
+      <c r="B7" s="38" t="n">
         <v>0.58</v>
       </c>
-      <c r="D7" s="33" t="s">
-        <v>236</v>
+      <c r="D7" s="37" t="s">
+        <v>240</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="B8" s="36" t="n">
+        <v>92</v>
+      </c>
+      <c r="B8" s="40" t="n">
         <f aca="false">1-B6</f>
         <v>0.5</v>
       </c>
-      <c r="D8" s="33" t="s">
-        <v>90</v>
+      <c r="D8" s="37" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>237</v>
-      </c>
-      <c r="B9" s="32" t="n">
+        <v>241</v>
+      </c>
+      <c r="B9" s="36" t="n">
         <v>4000</v>
       </c>
-      <c r="D9" s="33" t="s">
-        <v>238</v>
+      <c r="D9" s="37" t="s">
+        <v>242</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="B11" s="14"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>240</v>
-      </c>
-      <c r="B12" s="67" t="n">
+        <v>244</v>
+      </c>
+      <c r="B12" s="72" t="n">
         <f aca="false">B4*(1-B6)</f>
         <v>300000</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="B13" s="10" t="n">
         <f aca="false">B12/B5</f>
@@ -4070,7 +4126,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="B14" s="10" t="n">
         <f aca="false">B13*(1-B5)</f>
@@ -4079,7 +4135,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="B15" s="10" t="n">
         <f aca="false">B4*B6</f>
@@ -4088,31 +4144,31 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="B17" s="14"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="19" t="s">
-        <v>245</v>
-      </c>
-      <c r="B18" s="43" t="n">
+      <c r="A18" s="23" t="s">
+        <v>249</v>
+      </c>
+      <c r="B18" s="48" t="n">
         <f aca="false">B14*B7</f>
         <v>43500</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="19" t="s">
-        <v>218</v>
-      </c>
-      <c r="B19" s="43" t="n">
+      <c r="A19" s="23" t="s">
+        <v>222</v>
+      </c>
+      <c r="B19" s="48" t="n">
         <f aca="false">B15*B7</f>
         <v>174000</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="B20" s="10" t="n">
         <f aca="false">B18</f>
@@ -4121,7 +4177,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="B21" s="10" t="n">
         <f aca="false">B19</f>
@@ -4130,31 +4186,31 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="14" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="B23" s="14"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="19" t="s">
-        <v>249</v>
-      </c>
-      <c r="B24" s="43" t="n">
+      <c r="A24" s="23" t="s">
+        <v>253</v>
+      </c>
+      <c r="B24" s="48" t="n">
         <f aca="false">B9</f>
         <v>4000</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="19" t="s">
-        <v>223</v>
-      </c>
-      <c r="B25" s="43" t="n">
+      <c r="A25" s="23" t="s">
+        <v>227</v>
+      </c>
+      <c r="B25" s="48" t="n">
         <f aca="false">B4*B8</f>
         <v>300000</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="B26" s="10" t="n">
         <f aca="false">B24</f>
@@ -4163,7 +4219,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="B27" s="10" t="n">
         <f aca="false">B25</f>
@@ -4203,126 +4259,126 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="61" t="s">
-        <v>250</v>
-      </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
+      <c r="A1" s="66" t="s">
+        <v>254</v>
+      </c>
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="B3" s="14"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>251</v>
-      </c>
-      <c r="B4" s="32" t="n">
+        <v>255</v>
+      </c>
+      <c r="B4" s="36" t="n">
         <v>49500000</v>
       </c>
-      <c r="D4" s="33" t="s">
-        <v>252</v>
+      <c r="D4" s="37" t="s">
+        <v>256</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>253</v>
-      </c>
-      <c r="B5" s="32" t="n">
+        <v>257</v>
+      </c>
+      <c r="B5" s="36" t="n">
         <v>10500000</v>
       </c>
-      <c r="D5" s="33" t="s">
-        <v>254</v>
+      <c r="D5" s="37" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>255</v>
-      </c>
-      <c r="B6" s="32" t="n">
+        <v>259</v>
+      </c>
+      <c r="B6" s="36" t="n">
         <v>15900000</v>
       </c>
-      <c r="D6" s="33" t="s">
-        <v>256</v>
+      <c r="D6" s="37" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>257</v>
-      </c>
-      <c r="B7" s="32" t="n">
+        <v>261</v>
+      </c>
+      <c r="B7" s="36" t="n">
         <v>5000000</v>
       </c>
-      <c r="D7" s="33" t="s">
-        <v>258</v>
+      <c r="D7" s="37" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>259</v>
-      </c>
-      <c r="B8" s="34" t="n">
+        <v>263</v>
+      </c>
+      <c r="B8" s="38" t="n">
         <v>0.75</v>
       </c>
-      <c r="D8" s="33" t="s">
-        <v>260</v>
+      <c r="D8" s="37" t="s">
+        <v>264</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>261</v>
-      </c>
-      <c r="B9" s="34" t="n">
+        <v>265</v>
+      </c>
+      <c r="B9" s="38" t="n">
         <v>0.45</v>
       </c>
-      <c r="D9" s="33" t="s">
-        <v>262</v>
+      <c r="D9" s="37" t="s">
+        <v>266</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>263</v>
-      </c>
-      <c r="B10" s="32" t="n">
+        <v>267</v>
+      </c>
+      <c r="B10" s="36" t="n">
         <v>238381</v>
       </c>
-      <c r="D10" s="33" t="s">
-        <v>264</v>
+      <c r="D10" s="37" t="s">
+        <v>268</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="B13" s="14"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="19" t="s">
-        <v>265</v>
-      </c>
-      <c r="B14" s="43" t="n">
+      <c r="A14" s="23" t="s">
+        <v>269</v>
+      </c>
+      <c r="B14" s="48" t="n">
         <f aca="false">B7</f>
         <v>5000000</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="19" t="s">
-        <v>266</v>
-      </c>
-      <c r="B15" s="43" t="n">
+      <c r="A15" s="23" t="s">
+        <v>270</v>
+      </c>
+      <c r="B15" s="48" t="n">
         <f aca="false">B6*B8</f>
         <v>11925000</v>
       </c>
-      <c r="D15" s="33" t="s">
-        <v>267</v>
+      <c r="D15" s="37" t="s">
+        <v>271</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="16" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="B16" s="16"/>
       <c r="C16" s="16"/>
@@ -4330,7 +4386,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="B18" s="10" t="n">
         <f aca="false">B14</f>
@@ -4339,7 +4395,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="B19" s="10" t="n">
         <f aca="false">B15</f>
@@ -4348,31 +4404,31 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="14" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="B21" s="14"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="19" t="s">
-        <v>222</v>
-      </c>
-      <c r="B22" s="43" t="n">
+      <c r="A22" s="23" t="s">
+        <v>226</v>
+      </c>
+      <c r="B22" s="48" t="n">
         <f aca="false">B10</f>
         <v>238381</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="19" t="s">
-        <v>269</v>
-      </c>
-      <c r="B23" s="43" t="n">
+      <c r="A23" s="23" t="s">
+        <v>273</v>
+      </c>
+      <c r="B23" s="48" t="n">
         <f aca="false">B4*B9</f>
         <v>22275000</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="B24" s="10" t="n">
         <f aca="false">B22</f>
@@ -4381,7 +4437,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="B25" s="10" t="n">
         <f aca="false">B23</f>
@@ -4418,137 +4474,137 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="68" t="s">
-        <v>270</v>
+      <c r="A1" s="73" t="s">
+        <v>274</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="69" t="s">
-        <v>271</v>
+      <c r="A3" s="74" t="s">
+        <v>275</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="70" t="s">
-        <v>272</v>
+      <c r="A4" s="75" t="s">
+        <v>276</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="70" t="s">
-        <v>273</v>
+      <c r="A5" s="75" t="s">
+        <v>277</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="70"/>
+      <c r="A6" s="75"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="69" t="s">
-        <v>274</v>
+      <c r="A7" s="74" t="s">
+        <v>278</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="70" t="s">
-        <v>275</v>
+      <c r="A8" s="75" t="s">
+        <v>279</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="70" t="s">
-        <v>276</v>
+      <c r="A9" s="75" t="s">
+        <v>280</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="70" t="s">
-        <v>277</v>
+      <c r="A10" s="75" t="s">
+        <v>281</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="70"/>
+      <c r="A11" s="75"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="69" t="s">
-        <v>278</v>
+      <c r="A12" s="74" t="s">
+        <v>282</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="70" t="s">
-        <v>279</v>
+      <c r="A13" s="75" t="s">
+        <v>283</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="70" t="s">
-        <v>280</v>
+      <c r="A14" s="75" t="s">
+        <v>284</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="70" t="s">
-        <v>281</v>
+      <c r="A15" s="75" t="s">
+        <v>285</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="70" t="s">
-        <v>282</v>
+      <c r="A16" s="75" t="s">
+        <v>286</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="70"/>
+      <c r="A17" s="75"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="69" t="s">
-        <v>283</v>
+      <c r="A18" s="74" t="s">
+        <v>287</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="70" t="s">
-        <v>284</v>
+      <c r="A19" s="75" t="s">
+        <v>288</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="70" t="s">
-        <v>285</v>
+      <c r="A20" s="75" t="s">
+        <v>289</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="70" t="s">
-        <v>286</v>
+      <c r="A21" s="75" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="70" t="s">
-        <v>287</v>
+      <c r="A22" s="75" t="s">
+        <v>291</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="70" t="s">
-        <v>288</v>
+      <c r="A23" s="75" t="s">
+        <v>292</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="70" t="s">
-        <v>289</v>
+      <c r="A24" s="75" t="s">
+        <v>293</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="70" t="s">
-        <v>290</v>
+      <c r="A25" s="75" t="s">
+        <v>294</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="70" t="s">
-        <v>291</v>
+      <c r="A26" s="75" t="s">
+        <v>295</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="70" t="s">
-        <v>292</v>
+      <c r="A27" s="75" t="s">
+        <v>296</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="70" t="s">
-        <v>293</v>
+      <c r="A28" s="75" t="s">
+        <v>297</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="70" t="s">
-        <v>294</v>
+      <c r="A29" s="75" t="s">
+        <v>298</v>
       </c>
     </row>
   </sheetData>

</xml_diff>